<commit_message>
data: 更新 2026-02 (TT=179.937 Kwai=60.374)
</commit_message>
<xml_diff>
--- a/docs/data/巴西数据底稿_2026-02.xlsx
+++ b/docs/data/巴西数据底稿_2026-02.xlsx
@@ -532,7 +532,7 @@
         <v>19.61</v>
       </c>
       <c r="K2" t="n">
-        <v>129.48</v>
+        <v>129.49</v>
       </c>
       <c r="L2" t="n">
         <v>28.59</v>
@@ -1156,7 +1156,7 @@
         <v>4.189</v>
       </c>
       <c r="K74" t="n">
-        <v>66.654</v>
+        <v>66.66200000000001</v>
       </c>
       <c r="L74" t="n">
         <v>3.924</v>

</xml_diff>